<commit_message>
settings update and deck rebalance
</commit_message>
<xml_diff>
--- a/chozoreference.xlsx
+++ b/chozoreference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\polyc\Desktop\Project Files\legacyofchozo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A2232D-8E50-4E86-B2B1-837727F63214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5586B3B-D8F2-4C97-8962-1EE7D839B7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="2" xr2:uid="{E42863CE-C03E-44E5-940B-DCEC359E2BB6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{E42863CE-C03E-44E5-940B-DCEC359E2BB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="276">
   <si>
     <t>type</t>
   </si>
@@ -162,9 +162,6 @@
     <t>--</t>
   </si>
   <si>
-    <t>If this ship exhausts for containment, also ready one Galactic Federation character</t>
-  </si>
-  <si>
     <t>Chozo - Thoha</t>
   </si>
   <si>
@@ -546,9 +543,6 @@
     <t>@[ex]: Refund 1 CP the next time a "Bounty Hunter" character activates its ability</t>
   </si>
   <si>
-    <t>@[cost,1]@[ex]: Target ship has +1 Security this turn</t>
-  </si>
-  <si>
     <t>@[cost,1]: Ready target ship</t>
   </si>
   <si>
@@ -720,9 +714,6 @@
     <t>chozo_ghosts</t>
   </si>
   <si>
-    <t>Their aggressive and erratic behaviour is most likely due to the corrupting effects of Phazon in the Tallon IV environment.</t>
-  </si>
-  <si>
     <t>Hive Mind Communication</t>
   </si>
   <si>
@@ -874,6 +865,15 @@
   </si>
   <si>
     <t>At the end of each turn, move a Phazon token from another card you control to Chozo Ghosts. Then, if this card has 3 or more Phazon tokens, discard it and put its Phazon tokens on a character your opponent controls.</t>
+  </si>
+  <si>
+    <t>@[ex]: Select another ship you control that is being raided. If it is a Galactic Federation ship it gains 2 Security until end of turn, otherwise it gets 1</t>
+  </si>
+  <si>
+    <t>If this ship exhausts for containment, also ready one Galactic Federation character.\nWhen this ship is being raided, Galactic Federation characters contribute 1 more strength than normal.</t>
+  </si>
+  <si>
+    <t>When a ship you control is destroyed from a raid, if GF Soldier is ready, @[ex] it and your opponent's lowest stage Metroid breaches.</t>
   </si>
 </sst>
 </file>
@@ -1264,10 +1264,10 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1297,16 +1297,16 @@
         <v>16</v>
       </c>
       <c r="L1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="N1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="O1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -1314,7 +1314,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -1323,16 +1323,16 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G2" t="s">
         <v>20</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -1344,10 +1344,10 @@
         <v>3</v>
       </c>
       <c r="L2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="N2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O2">
         <v>2</v>
@@ -1358,7 +1358,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
@@ -1367,16 +1367,16 @@
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G3" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I3">
         <v>2</v>
@@ -1388,10 +1388,10 @@
         <v>3</v>
       </c>
       <c r="L3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="N3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -1402,7 +1402,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -1411,16 +1411,16 @@
         <v>4</v>
       </c>
       <c r="E4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" t="s">
         <v>81</v>
-      </c>
-      <c r="F4" t="s">
-        <v>82</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="I4">
         <v>2</v>
@@ -1432,10 +1432,10 @@
         <v>3</v>
       </c>
       <c r="L4" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="N4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O4">
         <v>2</v>
@@ -1446,10 +1446,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D5" t="s">
         <v>4</v>
@@ -1461,10 +1461,10 @@
         <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I5">
         <v>2</v>
@@ -1476,13 +1476,13 @@
         <v>3</v>
       </c>
       <c r="L5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="M5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -1493,7 +1493,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -1502,16 +1502,16 @@
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -1523,7 +1523,7 @@
         <v>2</v>
       </c>
       <c r="N6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O6">
         <v>4</v>
@@ -1534,7 +1534,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -1543,16 +1543,16 @@
         <v>4</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" t="s">
         <v>68</v>
-      </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" t="s">
-        <v>69</v>
       </c>
       <c r="I7">
         <v>2</v>
@@ -1564,10 +1564,10 @@
         <v>3</v>
       </c>
       <c r="L7" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="N7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O7">
         <v>2</v>
@@ -1578,7 +1578,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
@@ -1587,16 +1587,16 @@
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G8" t="s">
         <v>23</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -1608,7 +1608,7 @@
         <v>2</v>
       </c>
       <c r="N8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O8">
         <v>4</v>
@@ -1619,7 +1619,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
@@ -1637,7 +1637,7 @@
         <v>23</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="I9">
         <v>3</v>
@@ -1649,10 +1649,10 @@
         <v>4</v>
       </c>
       <c r="L9" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="N9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O9">
         <v>2</v>
@@ -1663,7 +1663,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
         <v>5</v>
@@ -1672,16 +1672,16 @@
         <v>4</v>
       </c>
       <c r="E10" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F10" t="s">
+        <v>187</v>
+      </c>
+      <c r="G10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="G10" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>191</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1693,7 +1693,7 @@
         <v>2</v>
       </c>
       <c r="N10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O10">
         <v>2</v>
@@ -1704,7 +1704,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
         <v>2</v>
@@ -1713,16 +1713,16 @@
         <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G11" t="s">
         <v>11</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>166</v>
+        <v>275</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -1734,7 +1734,7 @@
         <v>2</v>
       </c>
       <c r="N11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O11">
         <v>2</v>
@@ -1745,7 +1745,7 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
@@ -1754,16 +1754,16 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G12" t="s">
         <v>11</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I12">
         <v>1</v>
@@ -1775,10 +1775,10 @@
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="N12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O12">
         <v>4</v>
@@ -1789,7 +1789,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
         <v>2</v>
@@ -1798,16 +1798,16 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G13" t="s">
         <v>11</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I13">
         <v>2</v>
@@ -1819,10 +1819,10 @@
         <v>3</v>
       </c>
       <c r="L13" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="N13" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O13">
         <v>2</v>
@@ -1833,7 +1833,7 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C14" t="s">
         <v>2</v>
@@ -1851,7 +1851,7 @@
         <v>11</v>
       </c>
       <c r="H14" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I14">
         <v>2</v>
@@ -1863,10 +1863,10 @@
         <v>3</v>
       </c>
       <c r="L14" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="N14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O14">
         <v>2</v>
@@ -1877,7 +1877,7 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C15" t="s">
         <v>28</v>
@@ -1886,16 +1886,16 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
+        <v>100</v>
+      </c>
+      <c r="F15" t="s">
         <v>101</v>
-      </c>
-      <c r="F15" t="s">
-        <v>102</v>
       </c>
       <c r="G15" t="s">
         <v>32</v>
       </c>
       <c r="H15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I15" s="1">
         <v>0</v>
@@ -1907,10 +1907,10 @@
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N15" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O15">
         <v>2</v>
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
         <v>28</v>
@@ -1930,16 +1930,16 @@
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G16" t="s">
         <v>32</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -1951,7 +1951,7 @@
         <v>2</v>
       </c>
       <c r="N16" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O16">
         <v>4</v>
@@ -1962,7 +1962,7 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
         <v>3</v>
@@ -1971,19 +1971,19 @@
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G17" t="s">
         <v>26</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="I17" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J17">
         <v>3</v>
@@ -1992,10 +1992,10 @@
         <v>2</v>
       </c>
       <c r="L17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N17" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O17">
         <v>4</v>
@@ -2006,7 +2006,7 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C18" t="s">
         <v>3</v>
@@ -2015,16 +2015,16 @@
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G18" t="s">
         <v>26</v>
       </c>
       <c r="H18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I18">
         <v>2</v>
@@ -2036,10 +2036,10 @@
         <v>3</v>
       </c>
       <c r="L18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="N18" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O18">
         <v>2</v>
@@ -2050,7 +2050,7 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C19" t="s">
         <v>3</v>
@@ -2059,19 +2059,19 @@
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F19" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G19" t="s">
         <v>26</v>
       </c>
       <c r="H19" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I19" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J19">
         <v>6</v>
@@ -2080,10 +2080,10 @@
         <v>4</v>
       </c>
       <c r="L19" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="N19" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O19">
         <v>2</v>
@@ -2094,7 +2094,7 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
@@ -2103,22 +2103,22 @@
         <v>29</v>
       </c>
       <c r="E20" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F20" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G20" t="s">
         <v>29</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K20">
         <v>5</v>
       </c>
       <c r="N20" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O20">
         <v>4</v>
@@ -2129,7 +2129,7 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C21" t="s">
         <v>3</v>
@@ -2138,7 +2138,7 @@
         <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F21" t="s">
         <v>30</v>
@@ -2154,7 +2154,7 @@
         <v>5</v>
       </c>
       <c r="N21" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O21">
         <v>3</v>
@@ -2165,7 +2165,7 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C22" t="s">
         <v>28</v>
@@ -2174,22 +2174,22 @@
         <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G22" t="s">
         <v>29</v>
       </c>
       <c r="H22" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K22">
         <v>3</v>
       </c>
       <c r="N22" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O22">
         <v>3</v>
@@ -2200,7 +2200,7 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
         <v>28</v>
@@ -2209,19 +2209,19 @@
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F23" t="s">
+        <v>134</v>
+      </c>
+      <c r="G23" t="s">
         <v>135</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>136</v>
       </c>
-      <c r="H23" t="s">
-        <v>137</v>
-      </c>
       <c r="N23" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O23">
         <v>3</v>
@@ -2232,25 +2232,25 @@
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C24" t="s">
         <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J24">
         <v>4</v>
@@ -2259,7 +2259,7 @@
         <v>2</v>
       </c>
       <c r="N24" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O24">
         <v>2</v>
@@ -2270,25 +2270,25 @@
         <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
         <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F25" t="s">
+        <v>88</v>
+      </c>
+      <c r="G25" t="s">
         <v>89</v>
       </c>
-      <c r="G25" t="s">
-        <v>90</v>
-      </c>
       <c r="H25" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="J25">
         <v>4</v>
@@ -2297,7 +2297,7 @@
         <v>2</v>
       </c>
       <c r="N25" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O25">
         <v>2</v>
@@ -2308,25 +2308,25 @@
         <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C26" t="s">
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E26" t="s">
+        <v>95</v>
+      </c>
+      <c r="F26" t="s">
         <v>96</v>
-      </c>
-      <c r="F26" t="s">
-        <v>97</v>
       </c>
       <c r="G26" t="s">
         <v>11</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J26">
         <v>4</v>
@@ -2335,7 +2335,7 @@
         <v>2</v>
       </c>
       <c r="N26" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O26">
         <v>2</v>
@@ -2346,25 +2346,25 @@
         <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C27" t="s">
         <v>28</v>
       </c>
       <c r="D27" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" t="s">
+        <v>85</v>
+      </c>
+      <c r="F27" t="s">
         <v>84</v>
-      </c>
-      <c r="E27" t="s">
-        <v>86</v>
-      </c>
-      <c r="F27" t="s">
-        <v>85</v>
       </c>
       <c r="G27" t="s">
         <v>32</v>
       </c>
       <c r="H27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J27">
         <v>4</v>
@@ -2373,7 +2373,7 @@
         <v>2</v>
       </c>
       <c r="N27" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O27">
         <v>2</v>
@@ -2384,25 +2384,25 @@
         <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" t="s">
         <v>3</v>
       </c>
       <c r="D28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G28" t="s">
         <v>26</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J28">
         <v>4</v>
@@ -2411,7 +2411,7 @@
         <v>2</v>
       </c>
       <c r="N28" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O28">
         <v>2</v>
@@ -2422,25 +2422,25 @@
         <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
         <v>18</v>
       </c>
       <c r="D29" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
       </c>
       <c r="H29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I29">
         <v>3</v>
@@ -2452,7 +2452,7 @@
         <v>4</v>
       </c>
       <c r="N29" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O29">
         <v>2</v>
@@ -2463,26 +2463,26 @@
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C30" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E30" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" t="s">
+        <v>42</v>
+      </c>
+      <c r="G30" t="s">
+        <v>217</v>
+      </c>
+      <c r="H30" t="s">
         <v>44</v>
       </c>
-      <c r="F30" t="s">
-        <v>43</v>
-      </c>
-      <c r="G30" t="s">
-        <v>219</v>
-      </c>
-      <c r="H30" t="s">
-        <v>45</v>
-      </c>
       <c r="I30">
         <v>2</v>
       </c>
@@ -2493,10 +2493,10 @@
         <v>2</v>
       </c>
       <c r="M30" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O30">
         <v>4</v>
@@ -2507,25 +2507,25 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C31" t="s">
         <v>5</v>
       </c>
       <c r="D31" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I31">
         <v>3</v>
@@ -2537,7 +2537,7 @@
         <v>3</v>
       </c>
       <c r="N31" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O31">
         <v>3</v>
@@ -2548,25 +2548,25 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C32" t="s">
         <v>5</v>
       </c>
       <c r="D32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E32" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" t="s">
         <v>51</v>
-      </c>
-      <c r="F32" t="s">
-        <v>52</v>
       </c>
       <c r="G32" t="s">
         <v>23</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I32">
         <v>2</v>
@@ -2578,7 +2578,7 @@
         <v>3</v>
       </c>
       <c r="N32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O32">
         <v>3</v>
@@ -2589,25 +2589,25 @@
         <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C33" t="s">
         <v>2</v>
       </c>
       <c r="D33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E33" t="s">
+        <v>53</v>
+      </c>
+      <c r="F33" t="s">
         <v>54</v>
-      </c>
-      <c r="F33" t="s">
-        <v>55</v>
       </c>
       <c r="G33" t="s">
         <v>11</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>161</v>
+        <v>273</v>
       </c>
       <c r="I33">
         <v>2</v>
@@ -2619,7 +2619,7 @@
         <v>3</v>
       </c>
       <c r="N33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O33">
         <v>4</v>
@@ -2630,13 +2630,13 @@
         <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C34" t="s">
         <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E34" t="s">
         <v>7</v>
@@ -2648,7 +2648,7 @@
         <v>11</v>
       </c>
       <c r="H34" t="s">
-        <v>38</v>
+        <v>274</v>
       </c>
       <c r="I34">
         <v>4</v>
@@ -2660,7 +2660,7 @@
         <v>5</v>
       </c>
       <c r="N34" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O34">
         <v>2</v>
@@ -2671,16 +2671,16 @@
         <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
       </c>
       <c r="D35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E35" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="F35" t="s">
         <v>33</v>
@@ -2701,7 +2701,7 @@
         <v>1</v>
       </c>
       <c r="N35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O35">
         <v>4</v>
@@ -2712,19 +2712,19 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
       </c>
       <c r="D36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G36" t="s">
         <v>32</v>
@@ -2742,7 +2742,7 @@
         <v>3</v>
       </c>
       <c r="N36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O36">
         <v>2</v>
@@ -2753,16 +2753,16 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
       </c>
       <c r="D37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E37" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F37" t="s">
         <v>34</v>
@@ -2771,7 +2771,7 @@
         <v>32</v>
       </c>
       <c r="H37" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I37">
         <v>3</v>
@@ -2783,7 +2783,7 @@
         <v>4</v>
       </c>
       <c r="N37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O37">
         <v>2</v>
@@ -2794,25 +2794,25 @@
         <v>4</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C38" t="s">
         <v>3</v>
       </c>
       <c r="D38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E38" t="s">
+        <v>47</v>
+      </c>
+      <c r="F38" t="s">
         <v>48</v>
-      </c>
-      <c r="F38" t="s">
-        <v>49</v>
       </c>
       <c r="G38" t="s">
         <v>26</v>
       </c>
       <c r="H38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I38">
         <v>1</v>
@@ -2824,7 +2824,7 @@
         <v>1</v>
       </c>
       <c r="N38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O38">
         <v>4</v>
@@ -2835,25 +2835,25 @@
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C39" t="s">
         <v>3</v>
       </c>
       <c r="D39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G39" t="s">
         <v>26</v>
       </c>
       <c r="H39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I39">
         <v>3</v>
@@ -2865,7 +2865,7 @@
         <v>4</v>
       </c>
       <c r="N39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O39">
         <v>2</v>
@@ -2876,13 +2876,13 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C40" t="s">
         <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E40" t="s">
         <v>27</v>
@@ -2894,7 +2894,7 @@
         <v>26</v>
       </c>
       <c r="H40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I40">
         <v>4</v>
@@ -2906,7 +2906,7 @@
         <v>5</v>
       </c>
       <c r="N40" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O40">
         <v>2</v>
@@ -2917,25 +2917,25 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C41" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D41" t="s">
         <v>4</v>
       </c>
       <c r="E41" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F41" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="G41" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="I41">
         <v>0</v>
@@ -2947,13 +2947,13 @@
         <v>3</v>
       </c>
       <c r="L41" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="M41" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N41" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O41">
         <v>2</v>
@@ -2964,7 +2964,7 @@
         <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C42" t="s">
         <v>28</v>
@@ -2973,10 +2973,10 @@
         <v>4</v>
       </c>
       <c r="E42" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="F42" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G42" t="s">
         <v>32</v>
@@ -2991,10 +2991,10 @@
         <v>3</v>
       </c>
       <c r="L42" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N42" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O42">
         <v>2</v>
@@ -3005,19 +3005,19 @@
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C43" t="s">
         <v>28</v>
       </c>
       <c r="D43" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E43" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F43" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G43" t="s">
         <v>32</v>
@@ -3032,7 +3032,7 @@
         <v>2</v>
       </c>
       <c r="N43" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="O43">
         <v>3</v>
@@ -3043,7 +3043,7 @@
         <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C44" t="s">
         <v>28</v>
@@ -3052,22 +3052,22 @@
         <v>29</v>
       </c>
       <c r="E44" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F44" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G44" t="s">
         <v>29</v>
       </c>
       <c r="H44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K44">
         <v>2</v>
       </c>
       <c r="N44" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O44">
         <v>4</v>
@@ -3078,7 +3078,7 @@
         <v>4</v>
       </c>
       <c r="B45" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C45" t="s">
         <v>28</v>
@@ -3087,10 +3087,10 @@
         <v>4</v>
       </c>
       <c r="E45" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F45" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G45" t="s">
         <v>32</v>
@@ -3105,7 +3105,7 @@
         <v>2</v>
       </c>
       <c r="N45" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O45">
         <v>4</v>
@@ -3116,7 +3116,7 @@
         <v>2</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C46" t="s">
         <v>28</v>
@@ -3125,22 +3125,22 @@
         <v>29</v>
       </c>
       <c r="E46" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G46" t="s">
         <v>29</v>
       </c>
       <c r="H46" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K46">
         <v>2</v>
       </c>
       <c r="N46" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O46">
         <v>2</v>
@@ -3151,7 +3151,7 @@
         <v>2</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C47" t="s">
         <v>28</v>
@@ -3160,22 +3160,22 @@
         <v>29</v>
       </c>
       <c r="E47" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F47" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G47" t="s">
         <v>29</v>
       </c>
       <c r="H47" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K47">
         <v>2</v>
       </c>
       <c r="N47" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O47">
         <v>2</v>
@@ -3186,7 +3186,7 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C48" t="s">
         <v>28</v>
@@ -3195,22 +3195,22 @@
         <v>29</v>
       </c>
       <c r="E48" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F48" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G48" t="s">
         <v>29</v>
       </c>
       <c r="H48" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K48">
         <v>2</v>
       </c>
       <c r="N48" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="O48">
         <v>2</v>
@@ -3243,7 +3243,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -3273,13 +3273,13 @@
         <v>16</v>
       </c>
       <c r="L1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="N1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -3287,7 +3287,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
@@ -3296,10 +3296,10 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="F2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G2" t="s">
         <v>32</v>
@@ -3314,10 +3314,10 @@
         <v>3</v>
       </c>
       <c r="L2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="M2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N2">
         <f>A2</f>
@@ -3329,19 +3329,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
         <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E3" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G3" t="s">
         <v>32</v>
@@ -3356,7 +3356,7 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="N3">
         <f t="shared" ref="N3:N9" si="0">A3</f>
@@ -3368,7 +3368,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -3377,22 +3377,22 @@
         <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G4" t="s">
         <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K4">
         <v>2</v>
       </c>
       <c r="M4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N4">
         <f t="shared" si="0"/>
@@ -3404,7 +3404,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -3413,16 +3413,16 @@
         <v>4</v>
       </c>
       <c r="E5" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" t="s">
         <v>101</v>
-      </c>
-      <c r="F5" t="s">
-        <v>102</v>
       </c>
       <c r="G5" t="s">
         <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -3434,10 +3434,10 @@
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="M5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N5">
         <f t="shared" si="0"/>
@@ -3449,7 +3449,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
         <v>28</v>
@@ -3458,10 +3458,10 @@
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G6" t="s">
         <v>32</v>
@@ -3476,7 +3476,7 @@
         <v>2</v>
       </c>
       <c r="M6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
@@ -3488,7 +3488,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -3497,22 +3497,22 @@
         <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G7" t="s">
         <v>29</v>
       </c>
       <c r="H7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K7">
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N7">
         <f t="shared" si="0"/>
@@ -3524,7 +3524,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -3533,22 +3533,22 @@
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G8" t="s">
         <v>29</v>
       </c>
       <c r="H8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K8">
         <v>2</v>
       </c>
       <c r="M8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N8">
         <f t="shared" si="0"/>
@@ -3560,7 +3560,7 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
         <v>28</v>
@@ -3569,22 +3569,22 @@
         <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F9" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G9" t="s">
         <v>29</v>
       </c>
       <c r="H9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K9">
         <v>2</v>
       </c>
       <c r="M9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N9">
         <f t="shared" si="0"/>
@@ -3612,10 +3612,10 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -3645,16 +3645,16 @@
         <v>16</v>
       </c>
       <c r="L1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="N1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="O1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -3662,28 +3662,28 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>270</v>
+      </c>
+      <c r="F2" t="s">
         <v>199</v>
       </c>
-      <c r="C2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>273</v>
-      </c>
-      <c r="F2" t="s">
-        <v>201</v>
-      </c>
       <c r="G2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="I2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="J2">
         <v>5</v>
@@ -3692,10 +3692,10 @@
         <v>3</v>
       </c>
       <c r="M2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O2">
         <f t="shared" ref="O2:O11" si="0">A2</f>
@@ -3707,25 +3707,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C3" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D3" t="s">
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G3" t="s">
+        <v>200</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>204</v>
       </c>
       <c r="I3">
         <v>2</v>
@@ -3737,10 +3737,10 @@
         <v>3</v>
       </c>
       <c r="M3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O3">
         <f t="shared" si="0"/>
@@ -3752,25 +3752,25 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="I4">
         <v>2</v>
@@ -3782,7 +3782,7 @@
         <v>4</v>
       </c>
       <c r="N4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O4">
         <f t="shared" si="0"/>
@@ -3794,25 +3794,25 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C5" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="G5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -3824,7 +3824,7 @@
         <v>2</v>
       </c>
       <c r="N5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O5">
         <f t="shared" si="0"/>
@@ -3836,25 +3836,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E6" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="G6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I6">
         <v>4</v>
@@ -3866,10 +3866,10 @@
         <v>4</v>
       </c>
       <c r="M6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
@@ -3881,25 +3881,25 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>221</v>
+      </c>
+      <c r="F7" t="s">
+        <v>219</v>
+      </c>
+      <c r="G7" t="s">
         <v>220</v>
       </c>
-      <c r="D7" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" t="s">
-        <v>223</v>
-      </c>
-      <c r="F7" t="s">
-        <v>221</v>
-      </c>
-      <c r="G7" t="s">
-        <v>222</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -3910,14 +3910,11 @@
       <c r="K7">
         <v>2</v>
       </c>
-      <c r="L7" t="s">
-        <v>224</v>
-      </c>
       <c r="M7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O7">
         <f t="shared" si="0"/>
@@ -3929,31 +3926,31 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D8" t="s">
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="G8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="K8">
         <v>4</v>
       </c>
       <c r="N8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O8">
         <f t="shared" si="0"/>
@@ -3965,25 +3962,25 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C9" t="s">
+        <v>241</v>
+      </c>
+      <c r="D9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
+        <v>243</v>
+      </c>
+      <c r="F9" t="s">
+        <v>242</v>
+      </c>
+      <c r="G9" t="s">
         <v>244</v>
       </c>
-      <c r="D9" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="H9" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="F9" t="s">
-        <v>245</v>
-      </c>
-      <c r="G9" t="s">
-        <v>247</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>249</v>
       </c>
       <c r="I9">
         <v>3</v>
@@ -3995,13 +3992,13 @@
         <v>4</v>
       </c>
       <c r="L9" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="M9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O9">
         <f t="shared" si="0"/>
@@ -4013,7 +4010,7 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C10" t="s">
         <v>2</v>
@@ -4022,16 +4019,16 @@
         <v>4</v>
       </c>
       <c r="E10" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F10" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="G10" t="s">
         <v>11</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -4043,7 +4040,7 @@
         <v>3</v>
       </c>
       <c r="N10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O10">
         <f t="shared" si="0"/>
@@ -4055,31 +4052,31 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D11" t="s">
         <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="F11" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="G11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="K11">
         <v>4</v>
       </c>
       <c r="N11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="O11">
         <f t="shared" si="0"/>
@@ -4169,31 +4166,31 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B5">
         <f>SUM(Cards!A2:A100)</f>
@@ -4227,31 +4224,31 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B5">
         <f>SUM('Set2'!A2:A100)</f>
@@ -4274,34 +4271,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" t="s">
         <v>110</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>112</v>
       </c>
-      <c r="F1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G1" t="s">
-        <v>113</v>
-      </c>
       <c r="H1" t="s">
+        <v>118</v>
+      </c>
+      <c r="I1" t="s">
         <v>119</v>
       </c>
-      <c r="I1" t="s">
-        <v>120</v>
-      </c>
       <c r="J1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4309,13 +4306,13 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4327,7 +4324,7 @@
         <v>0.5</v>
       </c>
       <c r="I2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -4335,13 +4332,13 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4353,7 +4350,7 @@
         <v>1.5</v>
       </c>
       <c r="I3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -4361,13 +4358,13 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4379,7 +4376,7 @@
         <v>2</v>
       </c>
       <c r="I4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -4387,13 +4384,13 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4405,7 +4402,7 @@
         <v>4</v>
       </c>
       <c r="I5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -4413,13 +4410,13 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -4431,10 +4428,10 @@
         <v>6</v>
       </c>
       <c r="H6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -4442,16 +4439,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F7" s="1">
         <v>1</v>
@@ -4460,10 +4457,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="J7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -4478,15 +4475,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B2">
         <f>SUM(Starter!A2:A100)</f>

</xml_diff>